<commit_message>
Incluir a coluna de adiantamento salarial no resumo das três lojas
Coluna editável entre o adiantamento de incentivos e o vale-transporte,
como já existia nos relatórios de cada loja. O total de proventos, o
total de descontos e o líquido passam a ser fórmulas, para acompanhar o
que for digitado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RESUMO_3_LOJAS_AGOSTO_2026_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RESUMO_3_LOJAS_AGOSTO_2026_pgto_05-09-2026.xlsx
@@ -10,7 +10,7 @@
     <sheet name="RESUMO 3 LOJAS AGO.26" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RESUMO 3 LOJAS AGO.26'!$A$4:$O$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RESUMO 3 LOJAS AGO.26'!$A$4:$P$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00;-R$ #,##0.00;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,6 +66,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="00000000"/>
       <sz val="9"/>
@@ -94,7 +99,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -119,6 +124,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -158,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -174,23 +184,24 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -558,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -572,10 +583,11 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="70" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="70" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -650,20 +662,25 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
+          <t>ADIANTAMENTO SALARIAL / VALES</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
           <t>VALE TRANSP. 6%</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>TOTAL DESCONTOS</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>LÍQUIDO PARCIAL</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>OBSERVAÇÃO</t>
         </is>
@@ -689,6 +706,7 @@
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
+      <c r="P5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -720,22 +738,26 @@
       <c r="I6" s="7" t="n">
         <v>199</v>
       </c>
-      <c r="J6" s="8" t="n">
-        <v>5847.41</v>
+      <c r="J6" s="8">
+        <f>SUM(B6:I6)</f>
+        <v/>
       </c>
       <c r="K6" s="7" t="n">
         <v>-199</v>
       </c>
-      <c r="L6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="8" t="n">
-        <v>-199</v>
-      </c>
-      <c r="N6" s="9" t="n">
-        <v>5648.41</v>
-      </c>
-      <c r="O6" s="10" t="inlineStr">
+      <c r="L6" s="9" t="n"/>
+      <c r="M6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="8">
+        <f>SUM(K6:M6)</f>
+        <v/>
+      </c>
+      <c r="O6" s="10">
+        <f>J6+N6</f>
+        <v/>
+      </c>
+      <c r="P6" s="11" t="inlineStr">
         <is>
           <t>Não recebe comissão. Dia 15/08 trabalhado com folga compensatória.</t>
         </is>
@@ -771,22 +793,26 @@
       <c r="I7" s="7" t="n">
         <v>189</v>
       </c>
-      <c r="J7" s="8" t="n">
-        <v>5040.49</v>
+      <c r="J7" s="8">
+        <f>SUM(B7:I7)</f>
+        <v/>
       </c>
       <c r="K7" s="7" t="n">
         <v>-189</v>
       </c>
-      <c r="L7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="8" t="n">
-        <v>-189</v>
-      </c>
-      <c r="N7" s="9" t="n">
-        <v>4851.49</v>
-      </c>
-      <c r="O7" s="10" t="inlineStr">
+      <c r="L7" s="9" t="n"/>
+      <c r="M7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="8">
+        <f>SUM(K7:M7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="10">
+        <f>J7+N7</f>
+        <v/>
+      </c>
+      <c r="P7" s="11" t="inlineStr">
         <is>
           <t>Comissão fixa de R$ 2.000,00 (apurado R$ 909,51 + complemento R$ 1.090,49). 3 madrugadas = 24 h noturnas.</t>
         </is>
@@ -822,22 +848,26 @@
       <c r="I8" s="7" t="n">
         <v>73</v>
       </c>
-      <c r="J8" s="8" t="n">
-        <v>3402.06</v>
+      <c r="J8" s="8">
+        <f>SUM(B8:I8)</f>
+        <v/>
       </c>
       <c r="K8" s="7" t="n">
         <v>-73</v>
       </c>
-      <c r="L8" s="7" t="n">
+      <c r="L8" s="9" t="n"/>
+      <c r="M8" s="7" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="M8" s="8" t="n">
-        <v>-157.29</v>
-      </c>
-      <c r="N8" s="9" t="n">
-        <v>3244.77</v>
-      </c>
-      <c r="O8" s="10" t="inlineStr">
+      <c r="N8" s="8">
+        <f>SUM(K8:M8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="10">
+        <f>J8+N8</f>
+        <v/>
+      </c>
+      <c r="P8" s="11" t="inlineStr">
         <is>
           <t>24 horas extras. Adicional noturno fixo de R$ 350,00 — conferir com o ponto.</t>
         </is>
@@ -873,22 +903,26 @@
       <c r="I9" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="J9" s="8" t="n">
-        <v>145.18</v>
+      <c r="J9" s="8">
+        <f>SUM(B9:I9)</f>
+        <v/>
       </c>
       <c r="K9" s="7" t="n">
         <v>-22</v>
       </c>
-      <c r="L9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="8" t="n">
-        <v>-22</v>
-      </c>
-      <c r="N9" s="9" t="n">
-        <v>123.18</v>
-      </c>
-      <c r="O9" s="10" t="inlineStr">
+      <c r="L9" s="9" t="n"/>
+      <c r="M9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="8">
+        <f>SUM(K9:M9)</f>
+        <v/>
+      </c>
+      <c r="O9" s="10">
+        <f>J9+N9</f>
+        <v/>
+      </c>
+      <c r="P9" s="11" t="inlineStr">
         <is>
           <t>Férias de 01 a 31/08 pagas em recibo próprio (saiu em 04/08, volta em 04/09). Comissão dos dias 01 e 02/08.</t>
         </is>
@@ -924,22 +958,26 @@
       <c r="I10" s="7" t="n">
         <v>192</v>
       </c>
-      <c r="J10" s="8" t="n">
-        <v>3569.45</v>
+      <c r="J10" s="8">
+        <f>SUM(B10:I10)</f>
+        <v/>
       </c>
       <c r="K10" s="7" t="n">
         <v>-192</v>
       </c>
-      <c r="L10" s="7" t="n">
+      <c r="L10" s="9" t="n"/>
+      <c r="M10" s="7" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="M10" s="8" t="n">
-        <v>-276.29</v>
-      </c>
-      <c r="N10" s="9" t="n">
-        <v>3293.16</v>
-      </c>
-      <c r="O10" s="10" t="inlineStr">
+      <c r="N10" s="8">
+        <f>SUM(K10:M10)</f>
+        <v/>
+      </c>
+      <c r="O10" s="10">
+        <f>J10+N10</f>
+        <v/>
+      </c>
+      <c r="P10" s="11" t="inlineStr">
         <is>
           <t>Feriado 15/08 trabalhado. 2 madrugadas = 16 h noturnas, com folga no dia seguinte.</t>
         </is>
@@ -975,22 +1013,26 @@
       <c r="I11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="J11" s="8" t="n">
-        <v>2948.78</v>
+      <c r="J11" s="8">
+        <f>SUM(B11:I11)</f>
+        <v/>
       </c>
       <c r="K11" s="7" t="n">
         <v>-10</v>
       </c>
-      <c r="L11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="8" t="n">
-        <v>-10</v>
-      </c>
-      <c r="N11" s="9" t="n">
-        <v>2938.78</v>
-      </c>
-      <c r="O11" s="10" t="inlineStr">
+      <c r="L11" s="9" t="n"/>
+      <c r="M11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="8">
+        <f>SUM(K11:M11)</f>
+        <v/>
+      </c>
+      <c r="O11" s="10">
+        <f>J11+N11</f>
+        <v/>
+      </c>
+      <c r="P11" s="11" t="inlineStr">
         <is>
           <t>Comissão do Arraial (R$ 368,78) + loja Centro (R$ 2,65). Feriado 15/08 trabalhado.</t>
         </is>
@@ -1026,22 +1068,26 @@
       <c r="I12" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>1973.36</v>
+      <c r="J12" s="8">
+        <f>SUM(B12:I12)</f>
+        <v/>
       </c>
       <c r="K12" s="7" t="n">
         <v>-0</v>
       </c>
-      <c r="L12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="9" t="n">
-        <v>1973.36</v>
-      </c>
-      <c r="O12" s="10" t="inlineStr">
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="8">
+        <f>SUM(K12:M12)</f>
+        <v/>
+      </c>
+      <c r="O12" s="10">
+        <f>J12+N12</f>
+        <v/>
+      </c>
+      <c r="P12" s="11" t="inlineStr">
         <is>
           <t>1º mês completo após a admissão. Feriado 15/08 trabalhado.</t>
         </is>
@@ -1077,86 +1123,94 @@
       <c r="I13" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="8" t="n">
-        <v>2532.38</v>
+      <c r="J13" s="8">
+        <f>SUM(B13:I13)</f>
+        <v/>
       </c>
       <c r="K13" s="7" t="n">
         <v>-0</v>
       </c>
-      <c r="L13" s="7" t="n">
+      <c r="L13" s="9" t="n"/>
+      <c r="M13" s="7" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="M13" s="8" t="n">
-        <v>-84.29000000000001</v>
-      </c>
-      <c r="N13" s="9" t="n">
-        <v>2448.09</v>
-      </c>
-      <c r="O13" s="10" t="inlineStr">
+      <c r="N13" s="8">
+        <f>SUM(K13:M13)</f>
+        <v/>
+      </c>
+      <c r="O13" s="10">
+        <f>J13+N13</f>
+        <v/>
+      </c>
+      <c r="P13" s="11" t="inlineStr">
         <is>
           <t>17 horas extras noturnas (hora extra + adicional). Feriado 15/08 trabalhado.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>TOTAL ARRAIAL</t>
         </is>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="13">
         <f>SUM(B6:B13)</f>
         <v/>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="13">
         <f>SUM(C6:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="13">
         <f>SUM(D6:D13)</f>
         <v/>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="13">
         <f>SUM(E6:E13)</f>
         <v/>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="13">
         <f>SUM(F6:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="13">
         <f>SUM(G6:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="13">
         <f>SUM(H6:H13)</f>
         <v/>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="13">
         <f>SUM(I6:I13)</f>
         <v/>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="13">
         <f>SUM(J6:J13)</f>
         <v/>
       </c>
-      <c r="K14" s="12">
+      <c r="K14" s="13">
         <f>SUM(K6:K13)</f>
         <v/>
       </c>
-      <c r="L14" s="12">
+      <c r="L14" s="13">
         <f>SUM(L6:L13)</f>
         <v/>
       </c>
-      <c r="M14" s="12">
+      <c r="M14" s="13">
         <f>SUM(M6:M13)</f>
         <v/>
       </c>
-      <c r="N14" s="12">
+      <c r="N14" s="13">
         <f>SUM(N6:N13)</f>
         <v/>
       </c>
-      <c r="O14" s="13" t="n"/>
+      <c r="O14" s="13">
+        <f>SUM(O6:O13)</f>
+        <v/>
+      </c>
+      <c r="P14" s="14" t="n"/>
     </row>
     <row r="15" ht="19" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1178,6 +1232,7 @@
       <c r="M15" s="5" t="n"/>
       <c r="N15" s="5" t="n"/>
       <c r="O15" s="5" t="n"/>
+      <c r="P15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1209,22 +1264,26 @@
       <c r="I16" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="J16" s="8" t="n">
-        <v>5773.41</v>
+      <c r="J16" s="8">
+        <f>SUM(B16:I16)</f>
+        <v/>
       </c>
       <c r="K16" s="7" t="n">
         <v>-125</v>
       </c>
-      <c r="L16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="8" t="n">
-        <v>-125</v>
-      </c>
-      <c r="N16" s="9" t="n">
-        <v>5648.41</v>
-      </c>
-      <c r="O16" s="10" t="inlineStr">
+      <c r="L16" s="9" t="n"/>
+      <c r="M16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="8">
+        <f>SUM(K16:M16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="10">
+        <f>J16+N16</f>
+        <v/>
+      </c>
+      <c r="P16" s="11" t="inlineStr">
         <is>
           <t>Não recebe comissão.</t>
         </is>
@@ -1260,22 +1319,26 @@
       <c r="I17" s="7" t="n">
         <v>225</v>
       </c>
-      <c r="J17" s="8" t="n">
-        <v>3648.01</v>
+      <c r="J17" s="8">
+        <f>SUM(B17:I17)</f>
+        <v/>
       </c>
       <c r="K17" s="7" t="n">
         <v>-225</v>
       </c>
-      <c r="L17" s="7" t="n">
+      <c r="L17" s="9" t="n"/>
+      <c r="M17" s="7" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="M17" s="8" t="n">
-        <v>-309.29</v>
-      </c>
-      <c r="N17" s="9" t="n">
-        <v>3338.72</v>
-      </c>
-      <c r="O17" s="10" t="inlineStr"/>
+      <c r="N17" s="8">
+        <f>SUM(K17:M17)</f>
+        <v/>
+      </c>
+      <c r="O17" s="10">
+        <f>J17+N17</f>
+        <v/>
+      </c>
+      <c r="P17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1307,22 +1370,26 @@
       <c r="I18" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="8" t="n">
-        <v>0.74</v>
+      <c r="J18" s="8">
+        <f>SUM(B18:I18)</f>
+        <v/>
       </c>
       <c r="K18" s="7" t="n">
         <v>-0</v>
       </c>
-      <c r="L18" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="9" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="O18" s="10" t="inlineStr">
+      <c r="L18" s="9" t="n"/>
+      <c r="M18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="8">
+        <f>SUM(K18:M18)</f>
+        <v/>
+      </c>
+      <c r="O18" s="10">
+        <f>J18+N18</f>
+        <v/>
+      </c>
+      <c r="P18" s="11" t="inlineStr">
         <is>
           <t>Férias de 01 a 30/08 pagas em recibo próprio — conferir o dia 31/08.</t>
         </is>
@@ -1358,22 +1425,26 @@
       <c r="I19" s="7" t="n">
         <v>96</v>
       </c>
-      <c r="J19" s="8" t="n">
-        <v>2728.01</v>
+      <c r="J19" s="8">
+        <f>SUM(B19:I19)</f>
+        <v/>
       </c>
       <c r="K19" s="7" t="n">
         <v>-96</v>
       </c>
-      <c r="L19" s="7" t="n">
+      <c r="L19" s="9" t="n"/>
+      <c r="M19" s="7" t="n">
         <v>-74.29000000000001</v>
       </c>
-      <c r="M19" s="8" t="n">
-        <v>-170.29</v>
-      </c>
-      <c r="N19" s="9" t="n">
-        <v>2557.72</v>
-      </c>
-      <c r="O19" s="10" t="inlineStr"/>
+      <c r="N19" s="8">
+        <f>SUM(K19:M19)</f>
+        <v/>
+      </c>
+      <c r="O19" s="10">
+        <f>J19+N19</f>
+        <v/>
+      </c>
+      <c r="P19" s="11" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1405,22 +1476,26 @@
       <c r="I20" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="J20" s="8" t="n">
-        <v>1699.36</v>
+      <c r="J20" s="8">
+        <f>SUM(B20:I20)</f>
+        <v/>
       </c>
       <c r="K20" s="7" t="n">
         <v>-10</v>
       </c>
-      <c r="L20" s="7" t="n">
+      <c r="L20" s="9" t="n"/>
+      <c r="M20" s="7" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="M20" s="8" t="n">
-        <v>-94.29000000000001</v>
-      </c>
-      <c r="N20" s="9" t="n">
-        <v>1605.07</v>
-      </c>
-      <c r="O20" s="10" t="inlineStr"/>
+      <c r="N20" s="8">
+        <f>SUM(K20:M20)</f>
+        <v/>
+      </c>
+      <c r="O20" s="10">
+        <f>J20+N20</f>
+        <v/>
+      </c>
+      <c r="P20" s="11" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1452,86 +1527,94 @@
       <c r="I21" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="8" t="n">
-        <v>1621</v>
+      <c r="J21" s="8">
+        <f>SUM(B21:I21)</f>
+        <v/>
       </c>
       <c r="K21" s="7" t="n">
         <v>-0</v>
       </c>
-      <c r="L21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="9" t="n">
-        <v>1621</v>
-      </c>
-      <c r="O21" s="10" t="inlineStr">
+      <c r="L21" s="9" t="n"/>
+      <c r="M21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="8">
+        <f>SUM(K21:M21)</f>
+        <v/>
+      </c>
+      <c r="O21" s="10">
+        <f>J21+N21</f>
+        <v/>
+      </c>
+      <c r="P21" s="11" t="inlineStr">
         <is>
           <t>Não recebe comissão (apurado R$ 12,18 fica só como informação).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>TOTAL CENTRO</t>
         </is>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="13">
         <f>SUM(B16:B21)</f>
         <v/>
       </c>
-      <c r="C22" s="12">
+      <c r="C22" s="13">
         <f>SUM(C16:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="13">
         <f>SUM(D16:D21)</f>
         <v/>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="13">
         <f>SUM(E16:E21)</f>
         <v/>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="13">
         <f>SUM(F16:F21)</f>
         <v/>
       </c>
-      <c r="G22" s="12">
+      <c r="G22" s="13">
         <f>SUM(G16:G21)</f>
         <v/>
       </c>
-      <c r="H22" s="12">
+      <c r="H22" s="13">
         <f>SUM(H16:H21)</f>
         <v/>
       </c>
-      <c r="I22" s="12">
+      <c r="I22" s="13">
         <f>SUM(I16:I21)</f>
         <v/>
       </c>
-      <c r="J22" s="12">
+      <c r="J22" s="13">
         <f>SUM(J16:J21)</f>
         <v/>
       </c>
-      <c r="K22" s="12">
+      <c r="K22" s="13">
         <f>SUM(K16:K21)</f>
         <v/>
       </c>
-      <c r="L22" s="12">
+      <c r="L22" s="13">
         <f>SUM(L16:L21)</f>
         <v/>
       </c>
-      <c r="M22" s="12">
+      <c r="M22" s="13">
         <f>SUM(M16:M21)</f>
         <v/>
       </c>
-      <c r="N22" s="12">
+      <c r="N22" s="13">
         <f>SUM(N16:N21)</f>
         <v/>
       </c>
-      <c r="O22" s="13" t="n"/>
+      <c r="O22" s="13">
+        <f>SUM(O16:O21)</f>
+        <v/>
+      </c>
+      <c r="P22" s="14" t="n"/>
     </row>
     <row r="23" ht="19" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -1553,6 +1636,7 @@
       <c r="M23" s="5" t="n"/>
       <c r="N23" s="5" t="n"/>
       <c r="O23" s="5" t="n"/>
+      <c r="P23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1584,22 +1668,26 @@
       <c r="I24" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="J24" s="8" t="n">
-        <v>5673.41</v>
+      <c r="J24" s="8">
+        <f>SUM(B24:I24)</f>
+        <v/>
       </c>
       <c r="K24" s="7" t="n">
         <v>-25</v>
       </c>
-      <c r="L24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="8" t="n">
-        <v>-25</v>
-      </c>
-      <c r="N24" s="9" t="n">
-        <v>5648.41</v>
-      </c>
-      <c r="O24" s="10" t="inlineStr">
+      <c r="L24" s="9" t="n"/>
+      <c r="M24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="8">
+        <f>SUM(K24:M24)</f>
+        <v/>
+      </c>
+      <c r="O24" s="10">
+        <f>J24+N24</f>
+        <v/>
+      </c>
+      <c r="P24" s="11" t="inlineStr">
         <is>
           <t>Não recebe comissão.</t>
         </is>
@@ -1635,22 +1723,26 @@
       <c r="I25" s="7" t="n">
         <v>49</v>
       </c>
-      <c r="J25" s="8" t="n">
-        <v>3638.21</v>
+      <c r="J25" s="8">
+        <f>SUM(B25:I25)</f>
+        <v/>
       </c>
       <c r="K25" s="7" t="n">
         <v>-49</v>
       </c>
-      <c r="L25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="8" t="n">
-        <v>-49</v>
-      </c>
-      <c r="N25" s="9" t="n">
-        <v>3589.21</v>
-      </c>
-      <c r="O25" s="10" t="inlineStr">
+      <c r="L25" s="9" t="n"/>
+      <c r="M25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="8">
+        <f>SUM(K25:M25)</f>
+        <v/>
+      </c>
+      <c r="O25" s="10">
+        <f>J25+N25</f>
+        <v/>
+      </c>
+      <c r="P25" s="11" t="inlineStr">
         <is>
           <t>Comissão apurada R$ 825,38 × 2.</t>
         </is>
@@ -1686,22 +1778,26 @@
       <c r="I26" s="7" t="n">
         <v>260</v>
       </c>
-      <c r="J26" s="8" t="n">
-        <v>3994.48</v>
+      <c r="J26" s="8">
+        <f>SUM(B26:I26)</f>
+        <v/>
       </c>
       <c r="K26" s="7" t="n">
         <v>-260</v>
       </c>
-      <c r="L26" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="8" t="n">
-        <v>-260</v>
-      </c>
-      <c r="N26" s="9" t="n">
-        <v>3734.48</v>
-      </c>
-      <c r="O26" s="10" t="inlineStr">
+      <c r="L26" s="9" t="n"/>
+      <c r="M26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="8">
+        <f>SUM(K26:M26)</f>
+        <v/>
+      </c>
+      <c r="O26" s="10">
+        <f>J26+N26</f>
+        <v/>
+      </c>
+      <c r="P26" s="11" t="inlineStr">
         <is>
           <t>Comissão apurada R$ 886,30 × 2.</t>
         </is>
@@ -1737,22 +1833,26 @@
       <c r="I27" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J27" s="8" t="n">
-        <v>2709.49</v>
+      <c r="J27" s="8">
+        <f>SUM(B27:I27)</f>
+        <v/>
       </c>
       <c r="K27" s="7" t="n">
         <v>-0</v>
       </c>
-      <c r="L27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="9" t="n">
-        <v>2709.49</v>
-      </c>
-      <c r="O27" s="10" t="inlineStr">
+      <c r="L27" s="9" t="n"/>
+      <c r="M27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="8">
+        <f>SUM(K27:M27)</f>
+        <v/>
+      </c>
+      <c r="O27" s="10">
+        <f>J27+N27</f>
+        <v/>
+      </c>
+      <c r="P27" s="11" t="inlineStr">
         <is>
           <t>Comissão apurada R$ 235,42 × 2. 40 horas extras.</t>
         </is>
@@ -1788,252 +1888,272 @@
       <c r="I28" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J28" s="8" t="n">
-        <v>1920.46</v>
+      <c r="J28" s="8">
+        <f>SUM(B28:I28)</f>
+        <v/>
       </c>
       <c r="K28" s="7" t="n">
         <v>-0</v>
       </c>
-      <c r="L28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="9" t="n">
-        <v>1920.46</v>
-      </c>
-      <c r="O28" s="10" t="inlineStr">
+      <c r="L28" s="9" t="n"/>
+      <c r="M28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="8">
+        <f>SUM(K28:M28)</f>
+        <v/>
+      </c>
+      <c r="O28" s="10">
+        <f>J28+N28</f>
+        <v/>
+      </c>
+      <c r="P28" s="11" t="inlineStr">
         <is>
           <t>Comissão apurada R$ 125,58 × 2. Atestado de 02 a 08/09 é competência de setembro.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>TOTAL TRANCOSO</t>
         </is>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="13">
         <f>SUM(B24:B28)</f>
         <v/>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="13">
         <f>SUM(C24:C28)</f>
         <v/>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="13">
         <f>SUM(D24:D28)</f>
         <v/>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="13">
         <f>SUM(E24:E28)</f>
         <v/>
       </c>
-      <c r="F29" s="12">
+      <c r="F29" s="13">
         <f>SUM(F24:F28)</f>
         <v/>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="13">
         <f>SUM(G24:G28)</f>
         <v/>
       </c>
-      <c r="H29" s="12">
+      <c r="H29" s="13">
         <f>SUM(H24:H28)</f>
         <v/>
       </c>
-      <c r="I29" s="12">
+      <c r="I29" s="13">
         <f>SUM(I24:I28)</f>
         <v/>
       </c>
-      <c r="J29" s="12">
+      <c r="J29" s="13">
         <f>SUM(J24:J28)</f>
         <v/>
       </c>
-      <c r="K29" s="12">
+      <c r="K29" s="13">
         <f>SUM(K24:K28)</f>
         <v/>
       </c>
-      <c r="L29" s="12">
+      <c r="L29" s="13">
         <f>SUM(L24:L28)</f>
         <v/>
       </c>
-      <c r="M29" s="12">
+      <c r="M29" s="13">
         <f>SUM(M24:M28)</f>
         <v/>
       </c>
-      <c r="N29" s="12">
+      <c r="N29" s="13">
         <f>SUM(N24:N28)</f>
         <v/>
       </c>
-      <c r="O29" s="13" t="n"/>
+      <c r="O29" s="13">
+        <f>SUM(O24:O28)</f>
+        <v/>
+      </c>
+      <c r="P29" s="14" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>TOTAL GERAL — 3 LOJAS</t>
         </is>
       </c>
-      <c r="B31" s="15">
+      <c r="B31" s="16">
         <f>B14+B22+B29</f>
         <v/>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="16">
         <f>C14+C22+C29</f>
         <v/>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="16">
         <f>D14+D22+D29</f>
         <v/>
       </c>
-      <c r="E31" s="15">
+      <c r="E31" s="16">
         <f>E14+E22+E29</f>
         <v/>
       </c>
-      <c r="F31" s="15">
+      <c r="F31" s="16">
         <f>F14+F22+F29</f>
         <v/>
       </c>
-      <c r="G31" s="15">
+      <c r="G31" s="16">
         <f>G14+G22+G29</f>
         <v/>
       </c>
-      <c r="H31" s="15">
+      <c r="H31" s="16">
         <f>H14+H22+H29</f>
         <v/>
       </c>
-      <c r="I31" s="15">
+      <c r="I31" s="16">
         <f>I14+I22+I29</f>
         <v/>
       </c>
-      <c r="J31" s="15">
+      <c r="J31" s="16">
         <f>J14+J22+J29</f>
         <v/>
       </c>
-      <c r="K31" s="15">
+      <c r="K31" s="16">
         <f>K14+K22+K29</f>
         <v/>
       </c>
-      <c r="L31" s="15">
+      <c r="L31" s="16">
         <f>L14+L22+L29</f>
         <v/>
       </c>
-      <c r="M31" s="15">
+      <c r="M31" s="16">
         <f>M14+M22+M29</f>
         <v/>
       </c>
-      <c r="N31" s="15">
+      <c r="N31" s="16">
         <f>N14+N22+N29</f>
         <v/>
       </c>
-      <c r="O31" s="16" t="n"/>
+      <c r="O31" s="16">
+        <f>O14+O22+O29</f>
+        <v/>
+      </c>
+      <c r="P31" s="17" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>O QUE AINDA NÃO ESTÁ NESTE RESUMO — precisa ser somado antes de fechar o holerite:</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>• INSS e IRRF de cada funcionário (cálculo da contabilidade) — por isso a última coluna é LÍQUIDO PARCIAL.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="inlineStr">
-        <is>
-          <t>• Vales adiantados, convênio e descontos de falta do mês.</t>
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>• Convênio e descontos de falta do mês.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>• A coluna ADIANTAMENTO SALARIAL / VALES está em amarelo, para preencher com o valor adiantado a cada um (em negativo). O total de descontos e o líquido se atualizam sozinhos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>• Prêmio cota geral e prêmio pré-vencidos, conforme a apuração de metas de cada loja.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="18" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>• Diárias dos folguistas SERGIO (R$ 150,00) e ANA CELIA (R$ 100,00), na loja Centro — vão para o contas a pagar, fora do holerite.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="18" t="inlineStr"/>
-    </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="inlineStr">
         <is>
           <t>CRITÉRIOS USADOS:</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="19" t="inlineStr">
         <is>
           <t>• DSR sobre comissão e horas extras: 5 domingos ÷ 26 dias úteis de agosto/2026 = fator 0,192307.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="18" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>• Salário-hora = salário ÷ 220. Hora extra = salário-hora × 1,5 (R$ 11,0523). Adicional noturno = salário-hora × 20% (R$ 1,4736).</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="18" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>• Feriado de 15/08 trabalhado sem folga = 1 salário-dia a mais (R$ 54,03).</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="18" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>• TRANCOSO paga o dobro da comissão apurada no InovaFarma; os incentivos entram pelo valor simples.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="18" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>• Os incentivos são adiantados em dinheiro durante o mês, por isso aparecem como provento e como desconto (ADIANT. INCENT.).</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="18" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>• Comissões e incentivos vêm do relatório do InovaFarma de 01/08 a 31/08/2026, extraído em 03/09/2026.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O29"/>
-  <mergeCells count="15">
-    <mergeCell ref="A40:O40"/>
-    <mergeCell ref="A35:O35"/>
-    <mergeCell ref="A43:O43"/>
-    <mergeCell ref="A38:O38"/>
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A42:O42"/>
-    <mergeCell ref="A41:O41"/>
-    <mergeCell ref="A33:O33"/>
-    <mergeCell ref="A36:O36"/>
-    <mergeCell ref="A44:O44"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A37:O37"/>
-    <mergeCell ref="A45:O45"/>
-    <mergeCell ref="A34:O34"/>
-    <mergeCell ref="A39:O39"/>
+  <autoFilter ref="A4:P29"/>
+  <mergeCells count="16">
+    <mergeCell ref="A42:P42"/>
+    <mergeCell ref="A46:P46"/>
+    <mergeCell ref="A36:P36"/>
+    <mergeCell ref="A44:P44"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A37:P37"/>
+    <mergeCell ref="A40:P40"/>
+    <mergeCell ref="A45:P45"/>
+    <mergeCell ref="A39:P39"/>
+    <mergeCell ref="A34:P34"/>
+    <mergeCell ref="A35:P35"/>
+    <mergeCell ref="A38:P38"/>
+    <mergeCell ref="A43:P43"/>
+    <mergeCell ref="A41:P41"/>
+    <mergeCell ref="A33:P33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Incluir a coluna de férias pagas à parte no resumo das três lojas
Coluna editável depois do líquido, como lembrete para o contas a pagar:
recibo de férias pago fora do holerite, sem entrar no líquido.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RESUMO_3_LOJAS_AGOSTO_2026_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RESUMO_3_LOJAS_AGOSTO_2026_pgto_05-09-2026.xlsx
@@ -10,7 +10,7 @@
     <sheet name="RESUMO 3 LOJAS AGO.26" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RESUMO 3 LOJAS AGO.26'!$A$4:$P$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RESUMO 3 LOJAS AGO.26'!$A$4:$Q$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P46"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -587,7 +587,8 @@
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="70" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="70" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -681,6 +682,11 @@
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>FÉRIAS PAGAS À PARTE (contas a pagar)</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>OBSERVAÇÃO</t>
         </is>
@@ -707,6 +713,7 @@
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="5" t="n"/>
+      <c r="Q5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -757,7 +764,8 @@
         <f>J6+N6</f>
         <v/>
       </c>
-      <c r="P6" s="11" t="inlineStr">
+      <c r="P6" s="9" t="n"/>
+      <c r="Q6" s="11" t="inlineStr">
         <is>
           <t>Não recebe comissão. Dia 15/08 trabalhado com folga compensatória.</t>
         </is>
@@ -812,7 +820,8 @@
         <f>J7+N7</f>
         <v/>
       </c>
-      <c r="P7" s="11" t="inlineStr">
+      <c r="P7" s="9" t="n"/>
+      <c r="Q7" s="11" t="inlineStr">
         <is>
           <t>Comissão fixa de R$ 2.000,00 (apurado R$ 909,51 + complemento R$ 1.090,49). 3 madrugadas = 24 h noturnas.</t>
         </is>
@@ -867,7 +876,8 @@
         <f>J8+N8</f>
         <v/>
       </c>
-      <c r="P8" s="11" t="inlineStr">
+      <c r="P8" s="9" t="n"/>
+      <c r="Q8" s="11" t="inlineStr">
         <is>
           <t>24 horas extras. Adicional noturno fixo de R$ 350,00 — conferir com o ponto.</t>
         </is>
@@ -922,7 +932,8 @@
         <f>J9+N9</f>
         <v/>
       </c>
-      <c r="P9" s="11" t="inlineStr">
+      <c r="P9" s="9" t="n"/>
+      <c r="Q9" s="11" t="inlineStr">
         <is>
           <t>Férias de 01 a 31/08 pagas em recibo próprio (saiu em 04/08, volta em 04/09). Comissão dos dias 01 e 02/08.</t>
         </is>
@@ -977,7 +988,8 @@
         <f>J10+N10</f>
         <v/>
       </c>
-      <c r="P10" s="11" t="inlineStr">
+      <c r="P10" s="9" t="n"/>
+      <c r="Q10" s="11" t="inlineStr">
         <is>
           <t>Feriado 15/08 trabalhado. 2 madrugadas = 16 h noturnas, com folga no dia seguinte.</t>
         </is>
@@ -1032,7 +1044,8 @@
         <f>J11+N11</f>
         <v/>
       </c>
-      <c r="P11" s="11" t="inlineStr">
+      <c r="P11" s="9" t="n"/>
+      <c r="Q11" s="11" t="inlineStr">
         <is>
           <t>Comissão do Arraial (R$ 368,78) + loja Centro (R$ 2,65). Feriado 15/08 trabalhado.</t>
         </is>
@@ -1087,7 +1100,8 @@
         <f>J12+N12</f>
         <v/>
       </c>
-      <c r="P12" s="11" t="inlineStr">
+      <c r="P12" s="9" t="n"/>
+      <c r="Q12" s="11" t="inlineStr">
         <is>
           <t>1º mês completo após a admissão. Feriado 15/08 trabalhado.</t>
         </is>
@@ -1142,7 +1156,8 @@
         <f>J13+N13</f>
         <v/>
       </c>
-      <c r="P13" s="11" t="inlineStr">
+      <c r="P13" s="9" t="n"/>
+      <c r="Q13" s="11" t="inlineStr">
         <is>
           <t>17 horas extras noturnas (hora extra + adicional). Feriado 15/08 trabalhado.</t>
         </is>
@@ -1210,7 +1225,11 @@
         <f>SUM(O6:O13)</f>
         <v/>
       </c>
-      <c r="P14" s="14" t="n"/>
+      <c r="P14" s="13">
+        <f>SUM(P6:P13)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="14" t="n"/>
     </row>
     <row r="15" ht="19" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1233,6 +1252,7 @@
       <c r="N15" s="5" t="n"/>
       <c r="O15" s="5" t="n"/>
       <c r="P15" s="5" t="n"/>
+      <c r="Q15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1283,7 +1303,8 @@
         <f>J16+N16</f>
         <v/>
       </c>
-      <c r="P16" s="11" t="inlineStr">
+      <c r="P16" s="9" t="n"/>
+      <c r="Q16" s="11" t="inlineStr">
         <is>
           <t>Não recebe comissão.</t>
         </is>
@@ -1338,7 +1359,8 @@
         <f>J17+N17</f>
         <v/>
       </c>
-      <c r="P17" s="11" t="inlineStr"/>
+      <c r="P17" s="9" t="n"/>
+      <c r="Q17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1389,7 +1411,8 @@
         <f>J18+N18</f>
         <v/>
       </c>
-      <c r="P18" s="11" t="inlineStr">
+      <c r="P18" s="9" t="n"/>
+      <c r="Q18" s="11" t="inlineStr">
         <is>
           <t>Férias de 01 a 30/08 pagas em recibo próprio — conferir o dia 31/08.</t>
         </is>
@@ -1444,7 +1467,8 @@
         <f>J19+N19</f>
         <v/>
       </c>
-      <c r="P19" s="11" t="inlineStr"/>
+      <c r="P19" s="9" t="n"/>
+      <c r="Q19" s="11" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1495,7 +1519,8 @@
         <f>J20+N20</f>
         <v/>
       </c>
-      <c r="P20" s="11" t="inlineStr"/>
+      <c r="P20" s="9" t="n"/>
+      <c r="Q20" s="11" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1546,7 +1571,8 @@
         <f>J21+N21</f>
         <v/>
       </c>
-      <c r="P21" s="11" t="inlineStr">
+      <c r="P21" s="9" t="n"/>
+      <c r="Q21" s="11" t="inlineStr">
         <is>
           <t>Não recebe comissão (apurado R$ 12,18 fica só como informação).</t>
         </is>
@@ -1614,7 +1640,11 @@
         <f>SUM(O16:O21)</f>
         <v/>
       </c>
-      <c r="P22" s="14" t="n"/>
+      <c r="P22" s="13">
+        <f>SUM(P16:P21)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="14" t="n"/>
     </row>
     <row r="23" ht="19" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -1637,6 +1667,7 @@
       <c r="N23" s="5" t="n"/>
       <c r="O23" s="5" t="n"/>
       <c r="P23" s="5" t="n"/>
+      <c r="Q23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1687,7 +1718,8 @@
         <f>J24+N24</f>
         <v/>
       </c>
-      <c r="P24" s="11" t="inlineStr">
+      <c r="P24" s="9" t="n"/>
+      <c r="Q24" s="11" t="inlineStr">
         <is>
           <t>Não recebe comissão.</t>
         </is>
@@ -1742,7 +1774,8 @@
         <f>J25+N25</f>
         <v/>
       </c>
-      <c r="P25" s="11" t="inlineStr">
+      <c r="P25" s="9" t="n"/>
+      <c r="Q25" s="11" t="inlineStr">
         <is>
           <t>Comissão apurada R$ 825,38 × 2.</t>
         </is>
@@ -1797,7 +1830,8 @@
         <f>J26+N26</f>
         <v/>
       </c>
-      <c r="P26" s="11" t="inlineStr">
+      <c r="P26" s="9" t="n"/>
+      <c r="Q26" s="11" t="inlineStr">
         <is>
           <t>Comissão apurada R$ 886,30 × 2.</t>
         </is>
@@ -1852,7 +1886,8 @@
         <f>J27+N27</f>
         <v/>
       </c>
-      <c r="P27" s="11" t="inlineStr">
+      <c r="P27" s="9" t="n"/>
+      <c r="Q27" s="11" t="inlineStr">
         <is>
           <t>Comissão apurada R$ 235,42 × 2. 40 horas extras.</t>
         </is>
@@ -1907,7 +1942,8 @@
         <f>J28+N28</f>
         <v/>
       </c>
-      <c r="P28" s="11" t="inlineStr">
+      <c r="P28" s="9" t="n"/>
+      <c r="Q28" s="11" t="inlineStr">
         <is>
           <t>Comissão apurada R$ 125,58 × 2. Atestado de 02 a 08/09 é competência de setembro.</t>
         </is>
@@ -1975,7 +2011,11 @@
         <f>SUM(O24:O28)</f>
         <v/>
       </c>
-      <c r="P29" s="14" t="n"/>
+      <c r="P29" s="13">
+        <f>SUM(P24:P28)</f>
+        <v/>
+      </c>
+      <c r="Q29" s="14" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="15" t="inlineStr">
@@ -2039,7 +2079,11 @@
         <f>O14+O22+O29</f>
         <v/>
       </c>
-      <c r="P31" s="17" t="n"/>
+      <c r="P31" s="16">
+        <f>P14+P22+P29</f>
+        <v/>
+      </c>
+      <c r="Q31" s="17" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
@@ -2079,81 +2123,89 @@
     <row r="38">
       <c r="A38" s="19" t="inlineStr">
         <is>
+          <t>• A coluna FÉRIAS PAGAS À PARTE é só lembrete para o contas a pagar: recibo de férias pago fora do holerite, NÃO entra no líquido. Em agosto: JOEL (Arraial, férias de 01 a 31/08) e GENECIR (Centro, férias de 01 a 30/08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
           <t>• Diárias dos folguistas SERGIO (R$ 150,00) e ANA CELIA (R$ 100,00), na loja Centro — vão para o contas a pagar, fora do holerite.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="19" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="A40" s="20" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
         <is>
           <t>CRITÉRIOS USADOS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="19" t="inlineStr">
-        <is>
-          <t>• DSR sobre comissão e horas extras: 5 domingos ÷ 26 dias úteis de agosto/2026 = fator 0,192307.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>• Salário-hora = salário ÷ 220. Hora extra = salário-hora × 1,5 (R$ 11,0523). Adicional noturno = salário-hora × 20% (R$ 1,4736).</t>
+          <t>• DSR sobre comissão e horas extras: 5 domingos ÷ 26 dias úteis de agosto/2026 = fator 0,192307.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>• Feriado de 15/08 trabalhado sem folga = 1 salário-dia a mais (R$ 54,03).</t>
+          <t>• Salário-hora = salário ÷ 220. Hora extra = salário-hora × 1,5 (R$ 11,0523). Adicional noturno = salário-hora × 20% (R$ 1,4736).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="19" t="inlineStr">
         <is>
-          <t>• TRANCOSO paga o dobro da comissão apurada no InovaFarma; os incentivos entram pelo valor simples.</t>
+          <t>• Feriado de 15/08 trabalhado sem folga = 1 salário-dia a mais (R$ 54,03).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
         <is>
-          <t>• Os incentivos são adiantados em dinheiro durante o mês, por isso aparecem como provento e como desconto (ADIANT. INCENT.).</t>
+          <t>• TRANCOSO paga o dobro da comissão apurada no InovaFarma; os incentivos entram pelo valor simples.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
         <is>
+          <t>• Os incentivos são adiantados em dinheiro durante o mês, por isso aparecem como provento e como desconto (ADIANT. INCENT.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
           <t>• Comissões e incentivos vêm do relatório do InovaFarma de 01/08 a 31/08/2026, extraído em 03/09/2026.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P29"/>
-  <mergeCells count="16">
-    <mergeCell ref="A42:P42"/>
-    <mergeCell ref="A46:P46"/>
-    <mergeCell ref="A36:P36"/>
-    <mergeCell ref="A44:P44"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="A37:P37"/>
-    <mergeCell ref="A40:P40"/>
-    <mergeCell ref="A45:P45"/>
-    <mergeCell ref="A39:P39"/>
-    <mergeCell ref="A34:P34"/>
-    <mergeCell ref="A35:P35"/>
-    <mergeCell ref="A38:P38"/>
-    <mergeCell ref="A43:P43"/>
-    <mergeCell ref="A41:P41"/>
-    <mergeCell ref="A33:P33"/>
+  <autoFilter ref="A4:Q29"/>
+  <mergeCells count="17">
+    <mergeCell ref="A44:Q44"/>
+    <mergeCell ref="A40:Q40"/>
+    <mergeCell ref="A46:Q46"/>
+    <mergeCell ref="A39:Q39"/>
+    <mergeCell ref="A34:Q34"/>
+    <mergeCell ref="A35:Q35"/>
+    <mergeCell ref="A43:Q43"/>
+    <mergeCell ref="A38:Q38"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A42:Q42"/>
+    <mergeCell ref="A41:Q41"/>
+    <mergeCell ref="A33:Q33"/>
+    <mergeCell ref="A45:Q45"/>
+    <mergeCell ref="A47:Q47"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A37:Q37"/>
+    <mergeCell ref="A36:Q36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>